<commit_message>
Adding veteran to Intake record and moving veteran to after suicide referral flag in episode to make it consistent with Intake.
</commit_message>
<xml_diff>
--- a/doc/_static/example-files/PMHC-5-0-combined-delete.xlsx
+++ b/doc/_static/example-files/PMHC-5-0-combined-delete.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jennib/Work/git/PMHC/spec/doc/_static/example-files/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FD30D4E-80EA-FF45-A874-F6C9078F7B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="760" windowWidth="29800" windowHeight="17300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -29,12 +35,12 @@
     <sheet name="SIDAS" sheetId="20" r:id="rId20"/>
     <sheet name="WHO-5" sheetId="21" r:id="rId21"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="363">
   <si>
     <t>key</t>
   </si>
@@ -1128,8 +1134,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1166,13 +1172,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1210,7 +1224,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1244,6 +1258,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1278,9 +1293,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1453,11 +1469,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1465,7 +1481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1473,7 +1489,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1487,11 +1503,11 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1526,7 +1542,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1537,7 +1553,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1548,7 +1564,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1559,7 +1575,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1570,7 +1586,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1581,7 +1597,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1592,7 +1608,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1603,7 +1619,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1614,7 +1630,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1625,7 +1641,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1642,11 +1658,11 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:BC22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:55">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1813,7 +1829,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="2" spans="1:55">
+    <row r="2" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1824,7 +1840,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:55">
+    <row r="3" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1835,7 +1851,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:55">
+    <row r="4" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1846,7 +1862,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:55">
+    <row r="5" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1857,7 +1873,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:55">
+    <row r="6" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1868,7 +1884,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:55">
+    <row r="7" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1879,7 +1895,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:55">
+    <row r="8" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1890,7 +1906,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:55">
+    <row r="9" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1901,7 +1917,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:55">
+    <row r="10" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1912,7 +1928,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:55">
+    <row r="11" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1923,7 +1939,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:55">
+    <row r="12" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1934,7 +1950,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:55">
+    <row r="13" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -1945,7 +1961,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:55">
+    <row r="14" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1956,7 +1972,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:55">
+    <row r="15" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -1967,7 +1983,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:55">
+    <row r="16" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1978,7 +1994,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -1989,7 +2005,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -2000,7 +2016,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -2011,7 +2027,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -2022,7 +2038,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -2033,7 +2049,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -2050,11 +2066,11 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:T11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2116,7 +2132,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="2" spans="1:20">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2127,7 +2143,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2138,7 +2154,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:20">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2149,7 +2165,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:20">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2160,7 +2176,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:20">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2171,7 +2187,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:20">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2182,7 +2198,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:20">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2193,7 +2209,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:20">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2204,7 +2220,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:20">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2215,7 +2231,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:20">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2232,11 +2248,11 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2256,7 +2272,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2267,7 +2283,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2278,7 +2294,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2289,7 +2305,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2300,7 +2316,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2311,7 +2327,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2322,7 +2338,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2333,7 +2349,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2344,7 +2360,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2355,7 +2371,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2366,7 +2382,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -2377,7 +2393,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -2394,11 +2410,11 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2430,7 +2446,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2441,7 +2457,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2452,7 +2468,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2463,7 +2479,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2474,7 +2490,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2485,7 +2501,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2496,7 +2512,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2507,7 +2523,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2518,7 +2534,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2529,7 +2545,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2546,11 +2562,11 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2594,7 +2610,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2605,7 +2621,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2622,11 +2638,11 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2646,7 +2662,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2657,7 +2673,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2668,7 +2684,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2679,7 +2695,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2690,7 +2706,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2707,11 +2723,11 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2731,7 +2747,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2748,11 +2764,11 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2772,7 +2788,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2789,11 +2805,11 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2813,7 +2829,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2824,7 +2840,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2835,7 +2851,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2852,11 +2868,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2891,7 +2907,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2926,11 +2942,11 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2962,7 +2978,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2973,7 +2989,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2990,11 +3006,11 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3026,7 +3042,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3037,7 +3053,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3054,11 +3070,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3096,7 +3112,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3107,7 +3123,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3118,7 +3134,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3129,7 +3145,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3140,7 +3156,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3151,7 +3167,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -3168,11 +3184,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:P12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3207,19 +3223,22 @@
         <v>44</v>
       </c>
       <c r="L1" t="s">
+        <v>98</v>
+      </c>
+      <c r="M1" t="s">
         <v>45</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>46</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>47</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3230,7 +3249,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3241,7 +3260,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3252,7 +3271,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3263,7 +3282,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3274,7 +3293,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -3285,7 +3304,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3296,7 +3315,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -3307,7 +3326,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -3318,7 +3337,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -3329,7 +3348,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -3346,11 +3365,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:Q12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3403,7 +3422,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3414,7 +3433,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3425,7 +3444,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3436,7 +3455,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3447,7 +3466,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3458,7 +3477,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -3469,7 +3488,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3480,7 +3499,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -3491,7 +3510,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -3502,7 +3521,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -3513,7 +3532,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -3530,11 +3549,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AF11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:32">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3593,10 +3612,10 @@
         <v>97</v>
       </c>
       <c r="T1" t="s">
+        <v>44</v>
+      </c>
+      <c r="U1" t="s">
         <v>98</v>
-      </c>
-      <c r="U1" t="s">
-        <v>44</v>
       </c>
       <c r="V1" t="s">
         <v>99</v>
@@ -3632,7 +3651,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:32">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3643,7 +3662,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:32">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3654,7 +3673,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:32">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3665,7 +3684,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:32">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3676,7 +3695,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:32">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3687,7 +3706,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:32">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -3698,7 +3717,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:32">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3709,7 +3728,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:32">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -3720,7 +3739,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:32">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -3731,7 +3750,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:32">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -3748,11 +3767,11 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>118</v>
       </c>
@@ -3769,7 +3788,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3780,7 +3799,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3791,7 +3810,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3802,7 +3821,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3813,7 +3832,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3824,7 +3843,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -3835,7 +3854,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3846,7 +3865,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -3857,7 +3876,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -3868,7 +3887,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -3885,11 +3904,11 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3912,7 +3931,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3923,7 +3942,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3934,7 +3953,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3945,7 +3964,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3956,7 +3975,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3967,7 +3986,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -3978,7 +3997,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3989,7 +4008,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -4000,7 +4019,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -4011,7 +4030,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -4022,7 +4041,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -4033,7 +4052,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -4044,7 +4063,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -4055,7 +4074,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -4066,7 +4085,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -4077,7 +4096,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -4088,7 +4107,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -4099,7 +4118,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -4110,7 +4129,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -4121,7 +4140,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -4132,7 +4151,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -4149,11 +4168,11 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:T6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -4215,7 +4234,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:20">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -4226,7 +4245,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -4237,7 +4256,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:20">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -4248,7 +4267,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:20">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -4259,7 +4278,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:20">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>

</xml_diff>